<commit_message>
Aggiunto archetipo egizio "Piaghe"
</commit_message>
<xml_diff>
--- a/Holy War.xlsx
+++ b/Holy War.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\Holy-War-Python-Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0138A3A1-D155-45D3-A06C-AD0059E8DE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194294E8-D762-4C6A-93FD-65E9EBEA6F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="619">
   <si>
     <t>Nome Carta</t>
   </si>
@@ -1869,9 +1869,6 @@
     <t>Piaga: Zanzare del Deserto</t>
   </si>
   <si>
-    <t>Ogni Santo avversario perde 1 Fede. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
     <t>Piaga: Mosche d'Egitto</t>
   </si>
   <si>
@@ -1881,9 +1878,6 @@
     <t>Piaga: Ulcere della Carne</t>
   </si>
   <si>
-    <t>Scegli fino a 2 Santi avversari: ognuno perde 3 Fede. Poi infliggi 2 Peccato all'avversario. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
     <t>Piaga: Grandine di Fuoco</t>
   </si>
   <si>
@@ -1897,6 +1891,18 @@
   </si>
   <si>
     <t>Una volta per turno, quando questa carta attacca un Santo avversario, puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
+  </si>
+  <si>
+    <t>Portatore delle Piaghe</t>
+  </si>
+  <si>
+    <t>Ogni Santo avversario perde 3 Fede. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
+  </si>
+  <si>
+    <t>Scegli fino a 2 Santi avversari: ognuno perde 4 Fede. Poi infliggi 2 Peccato all'avversario. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
+  </si>
+  <si>
+    <t>Questa carta può essere evocata solo scomunicando 3 carte Piaga dalla tua mano o cimitero, senza pagare costo di Ispirazione. Questa carta non può essere bersagliata dagli effetti di altre carte. Una volta per turno, scegli e attiva un effetto di qualsiasi carta "Piaga" benedizione o maledizione.</t>
   </si>
 </sst>
 </file>
@@ -3397,8 +3403,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AD0662AD-6111-47FB-A32E-E5214BB172BE}" name="Tabella4" displayName="Tabella4" ref="A1:G57" totalsRowShown="0" headerRowDxfId="69" dataDxfId="67" headerRowBorderDxfId="68">
-  <autoFilter ref="A1:G57" xr:uid="{AD0662AD-6111-47FB-A32E-E5214BB172BE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AD0662AD-6111-47FB-A32E-E5214BB172BE}" name="Tabella4" displayName="Tabella4" ref="A1:G58" totalsRowShown="0" headerRowDxfId="69" dataDxfId="67" headerRowBorderDxfId="68">
+  <autoFilter ref="A1:G58" xr:uid="{AD0662AD-6111-47FB-A32E-E5214BB172BE}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{6899A739-52B8-45B2-B22F-D77E240FA270}" name="Nome Carta" dataDxfId="66"/>
     <tableColumn id="2" xr3:uid="{F5DF84CC-A246-40FD-980E-E7E55E602B3A}" name="Tipo" dataDxfId="65"/>
@@ -11166,7 +11172,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
@@ -12225,7 +12231,7 @@
         <v>6</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>167</v>
@@ -12282,7 +12288,7 @@
       <c r="D53" s="8"/>
       <c r="E53" s="8"/>
       <c r="F53" s="12" t="s">
-        <v>607</v>
+        <v>616</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>167</v>
@@ -12290,7 +12296,7 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>15</v>
@@ -12301,7 +12307,7 @@
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
       <c r="F54" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>167</v>
@@ -12309,7 +12315,7 @@
     </row>
     <row r="55" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>15</v>
@@ -12320,7 +12326,7 @@
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
       <c r="F55" s="12" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="G55" s="8" t="s">
         <v>167</v>
@@ -12328,7 +12334,7 @@
     </row>
     <row r="56" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>15</v>
@@ -12339,7 +12345,7 @@
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
       <c r="F56" s="12" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>167</v>
@@ -12347,7 +12353,7 @@
     </row>
     <row r="57" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>15</v>
@@ -12358,955 +12364,35 @@
       <c r="D57" s="8"/>
       <c r="E57" s="8"/>
       <c r="F57" s="12" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="10" t="s">
+        <v>615</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D58" s="8">
+        <v>25</v>
+      </c>
+      <c r="E58" s="8">
+        <v>10</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>618</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Pre once per turn piaga
</commit_message>
<xml_diff>
--- a/Holy War.xlsx
+++ b/Holy War.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\Holy-War-Python-Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194294E8-D762-4C6A-93FD-65E9EBEA6F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A5464C-CE41-4223-B4F5-E83F3AAD71ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -924,9 +924,6 @@
     <t>Finche questa carta è presente sul terreno, i tuoi Santi sono immuni agli effetti delle maledizioni.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ogni volta che un Token o un Santo viene mandato dal campo al cimitero, questo santo riceve +1 Fede e +1 Forza.</t>
-  </si>
-  <si>
     <t>Se questo Santo viene sconfitto da un Santo avversario, puoi prendere ogni carta "Pietra" dal tuo cimitero e metterla nel tuo reliquiario. Poi mischia il reliquiario. Se attivi questo effetto, scomunica questa carta.</t>
   </si>
   <si>
@@ -942,42 +939,24 @@
     <t>Ogni volta che questo Santo subisce danno non mortale, riceve +7 Fede.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ogni volta che un tuo Santo viene distrutto o giochi una carta "Sigillo", aggiungi 1 Segnalino Sigillo su questa carta. Puoi rimuovere un numero di Segnalini Sigillo pari alle Croci di una carta (tua o avversaria) il cui effetto sta per distruggere questa carta: annulla quell'effetto e questa carta non viene distrutta. Quando questa carta lascia il campo, rimuovi tutti i Segnalini Sigillo presenti su di essa.</t>
-  </si>
-  <si>
     <t>Quando questo Santo attacca un Santo avversario, dopo il calcolo del danno, equipaggia questa carta a quel Santo. Alla fine del prossimo turno, distruggi il Santo equipaggiato e scomunica questa carta.</t>
   </si>
   <si>
     <t>Quando questa carta lascia il campo, evoca un Token Spirito Vacuo sul tuo campo.</t>
   </si>
   <si>
-    <t>Puoi mandare questa carta dal campo al cimitero: evoca un qualsiasi Santo bersaglio dal tuo cimitero in zona d'attacco.</t>
-  </si>
-  <si>
-    <t>Se questo Santo distrugge un Santo con un attacco, torna nella tua mano. L'effetto di questa carta può essere attivato una volta per turno.</t>
-  </si>
-  <si>
     <t>Se Altare dei Sette Sigilli è sul campo con almeno 7 Segnalini Sigillo, questo Santo riceve +5 Forza. Quando questo Santo viene sconfitto in battaglia o distrutto per effetto di una carta, aggiungi 3 Segnalini Sigillo su Altare dei Sette Sigilli.</t>
   </si>
   <si>
     <t>Scegli due Santi sul campo. Distruggi tutti gli altri Santi.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ricevi +1 Ispirazione in questo turno.</t>
-  </si>
-  <si>
     <t>Scegli una carta Santo dal tuo cimitero e aggiungila alla tua mano.</t>
   </si>
   <si>
     <t>Gioca questa carta solo se 3 o più tuoi Santi sono stati mandati dalla tua mano o dal campo al cimitero in questo turno. Evoca "Fenrir" o "Jormungandr" dal tuo reliquiario o cimitero sul tuo campo.</t>
   </si>
   <si>
-    <t>Puoi giocare questa carta senza pagare il suo costo di Ispirazione. Finche questa carta è sul terreno, puoi giocare i Santi dalla tua mano pagando metà del loro costo di Ispirazione (arrotondato per eccesso).</t>
-  </si>
-  <si>
-    <t>Finche questo edificio è sul terreno, ogni volta che l'avversario pesca una carta, questa carta perde 1 Fede e rimuovi 2 Peccato da te stesso. Se la Fede di questa carta diventa 0, distruggi Av'drna.</t>
-  </si>
-  <si>
     <t>Ogni giocatore pesca 3 carte.</t>
   </si>
   <si>
@@ -990,18 +969,9 @@
     <t>Equipaggia questa carta a un Santo bersaglio. Quando la Fede di quel Santo diventa 0, puoi distruggere questa carta: quel Santo rimane con 1 Fede invece di essere sconfitto.</t>
   </si>
   <si>
-    <t>Finche questo edificio è sul tuo terreno, ogni volta che giochi una Benedizione o una Maledizione, aggiungi 1 Segnalino su questa carta. Puoi rimuovere 3 Segnalini da questa carta: cerca nel tuo reliquiario una Benedizione o Maledizione, rivelala e aggiungila alla tua mano. Poi mischia il reliquiario.</t>
-  </si>
-  <si>
-    <t>Finche questo edificio è sul tuo terreno, ogni volta che giochi una Benedizione, pesca una carta. Se è un Santo, scomunica quella carta. Se è un Artefatto o Edificio, rimetti quella carta nel tuo reliquiario e mischia. Se è una Benedizione o Maledizione, tienila in mano.</t>
-  </si>
-  <si>
     <t>Scomunica un Santo bersaglio, poi infliggi Peccato all'avversario pari alla Fede di quel Santo.</t>
   </si>
   <si>
-    <t>Per giocare questa carta, scegli un santo bersaglio sul tuo terreno e distruggilo. Successivamente, aggiungi la Fede iniziale del Santo sacrificato alla Fede di questa carta. Quando questo Santo viene sconfitto in battaglia o distrutto per effetto di una carta non genera Peccato.</t>
-  </si>
-  <si>
     <t>All'inizio del tuo turno, paga 5 Peccato, altrimenti distruggi questa carta. Alla fine del tuo turno, distruggi ogni tuo Token Spirito Vacuo. L'avversario riceve 5 Peccato per ogni Token distrutto in questo modo.</t>
   </si>
   <si>
@@ -1011,21 +981,6 @@
     <t>Mentre Campana è sul tuo terreno, all'inizio del tuo turno, aggiungi su di essa 1 Segnalino. Puoi attivare l'effetto di questa carta rimuovendo un qualsiasi numero di Segnalini da essa. Il costo in Ispirazione per attivare questo effetto è pari al numero di Segnalini rimossi. Per ogni Segnalino rimosso, ogni tuo Santo sul campo riceve +1 Fede.</t>
   </si>
   <si>
-    <t>Finche quesa carta è sul terreno, una volta per turno, scegli uno dei seguenti effetti: • Prendi un Santo dal tuo cimitero e aggiungilo alla tua mano, poi distruggi questa carta. • Se non controlli Santi, annulla il primo attacco che ricevi durante il prossimo turno avversario.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, prima della tua fase di pescata, devi distruggere un Santo bersaglio sul campo. Se hai distrutto un tuo Santo, infliggi 2 Peccato all'avversario. Se hai distrutto un Santo avversario, rimuovi 1 Peccato. Se, durante l'attivazione di questo effetto non sono presenti santi sul terreno, distruggi questa carta.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, ogni carta "Pietra" distrutta viene messa nel reliquiario del suo proprietario invece che nel cimitero.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, una volta per turno, puoi distruggere un tuo Santo bersaglio. Rimuovi Peccato pari alla Fede di quel Santo al momento della distruzione.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, ogni volta che peschi una carta, ogni tuo Santo sul campo riceve +2 Fede.</t>
-  </si>
-  <si>
     <t>Una volta per turno, scegli una carta Santo con Croci pari o inferiori a 4 nel tuo cimitero. Evoca quel Santo sul tuo campo senza pagare il suo costo di Ispirazione.</t>
   </si>
   <si>
@@ -1056,9 +1011,6 @@
     <t>Manda tutte le carte dalla tua mano al cimitero. Poi pesca 5 carte.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ogni volta che un Token Albero viene sconfitto, infliggi 1 Peccato all'avversario.</t>
-  </si>
-  <si>
     <t>Tre tuoi Santi bersaglio ricevono +5 Fede ciascuno.</t>
   </si>
   <si>
@@ -1068,9 +1020,6 @@
     <t>Per giocare questa carta, devi scomunicare dal tuo cimitero una copia di "Giorno 1", "Giorno 2", "Giorno 3", "Giorno 4", "Giorno 5", "Giorno 6" e "Giorno 7". Questa carta non può essere bersagliata da effetti.</t>
   </si>
   <si>
-    <t>Quando questo santo entra in campo, guarda la prima carta del tuo reliquiario. Se è una Benedizione o Maledizione, pescala. Altrimenti, rimischia il reliquiario.</t>
-  </si>
-  <si>
     <t>Cerca fino a 3 carte Albero nel tuo reliquiario e mandale al cimitero.</t>
   </si>
   <si>
@@ -1083,39 +1032,18 @@
     <t>Puoi pescare fino a 5 carte. Ogni carta pescata in questo modo costa 2 Ispirazione in questo turno.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ogni volta che un tuo Santo viene mandato al cimitero, evoca un Token Spirito Vacuo sul suo posto.</t>
-  </si>
-  <si>
     <t>Prendi il controllo di un tuo Santo e spostalo sul campo dell'avversario fino alla fine del turno. Quando quel Santo viene sconfitto, il giocatore che lo controlla in quel momento riceve Peccato pari alla sua Fede iniziale.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, durante la tua fase di pescata, pesca una carta aggiuntiva.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, una volta per turno, quando l'avversario pesca una carta, puoi fargli rimischiare quella carta nel reliquiario e pescare di nuovo.</t>
-  </si>
-  <si>
     <t>Ogni volta che questo Santo dichiara un attacco ad un Santo avversario, prima del calcolo del danno, riceve +1 Forza.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ogni volta che un Santo avversario attacca, subisce 2 danni. Se un Santo avversario viene distrutto da questo effetto, rimuovi 2 Peccato.</t>
-  </si>
-  <si>
     <t>Un Santo bersaglio riceve +3 Forza. Se controlli Odino, quel Santo riceve +6 Forza invece. Se controlli Odino e Thor, quel Santo riceve +6 Forza e peschi una carta.</t>
   </si>
   <si>
     <t>Ogni Santo con espansione "Animismo" sul tuo campo riceve +2 Fede e +2 Forza.</t>
   </si>
   <si>
-    <t>Finche questa carta è sul terreno, ogni carta che passa dal tuo campo direttamente al cimitero viene invece aggiunta alla tua mano.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, le tue carte Albero non possono essere bersagliate da Maledizioni o Benedizioni avversarie. Se una carta Albero viene scomunicata, viene messa nel reliquiario del suo proprietario invece che nella zona scomunicate.</t>
-  </si>
-  <si>
-    <t>Finche questa carta è sul terreno, una volta per turno puoi scomunicare la carta in cima al tuo reliquiario.</t>
-  </si>
-  <si>
     <t>Fino a quando questo Santo è sul campo, ogni volta che l'avversario pesca una carta, ogni tuo Santo sul campo riceve +1 Fede.</t>
   </si>
   <si>
@@ -1143,9 +1071,6 @@
     <t>I Santi avversari con Croci pari o inferiori a 2 non possono attaccare.</t>
   </si>
   <si>
-    <t>Rendi inutilizzabile uno slot Artefatto dell'avversario a tua scelta.</t>
-  </si>
-  <si>
     <t>Puoi giocare una carta Artefatto dalla tua mano pagando metà del suo costo di Ispirazione (arrotondato per eccesso).</t>
   </si>
   <si>
@@ -1173,9 +1098,6 @@
     <t>Prendi tutte le carte da tutti i cimiteri e rimettile nei rispettivi reliquiari. Poi ogni giocatore mischia il proprio reliquiario.</t>
   </si>
   <si>
-    <t>Se questo Santo distrugge un Santo avversario, aumenta la sua Fede a 4.</t>
-  </si>
-  <si>
     <t>Quando questa carta entra in campo, puoi evocare un Token Gub-ner sul tuo campo. Ogni volta che un Token Gub-ner viene sconfitto, puoi scegliere una carta scomunicata e rimetterla nel reliquiario del suo proprietario. Poi mischia.</t>
   </si>
   <si>
@@ -1188,9 +1110,6 @@
     <t>Quando giochi questo santo mentre Odino è presente sul tuo terreno, guarda le prime 3 carte del tuo reliquiario. Puoi aggiungere una qualsiasi di quelle carte alla tua mano e successivamente mischiare il reliquiario.</t>
   </si>
   <si>
-    <t>Per ogni 5 carte nel tuo cimitero, questa carta riceve +2 Fede e +2 Forza.</t>
-  </si>
-  <si>
     <t>Se non controlli altri Santi, puoi giocare questa carta senza pagare il suo costo di Ispirazione.</t>
   </si>
   <si>
@@ -1623,9 +1542,6 @@
     <t>Guarda la carta in fondo al tuo reliquiario. Puoi spostarla in cima o lasciarla in fondo.</t>
   </si>
   <si>
-    <t>Puoi includere questa carta solo in un reliquiario composto interamente da carte con espansione Ph-Dak'Gaph. Ogni volta che un giocatore pesca una carta riceve 1 peccato. Ogni volta che una carta viene scomunicata, perdi 1 peccato.</t>
-  </si>
-  <si>
     <t>Distruggi un Santo sul terreno dell'avversario.</t>
   </si>
   <si>
@@ -1647,9 +1563,6 @@
     <t>Questa carta può essere evocata solo tramite "Specchio di Ykknødar". Non può essere distrutta da effetti. Non può attaccare. Ogni volta che l'avversario pesca una carta, rimuovi 3 Peccato.</t>
   </si>
   <si>
-    <t>Manda una santo bersaglio dal tuo deck al cimitero. Rimuovi peccato pari alla fede e forza di quel santo.</t>
-  </si>
-  <si>
     <t>Cerca un artefatto nel tuo reliquiario o cimitero e posizionalo sul terreno senza pagare ispirazione.</t>
   </si>
   <si>
@@ -1659,39 +1572,15 @@
     <t>Una volta per turno, puoi distruggere un Token Gub-ner sul tuo terreno. Se lo fai, seleziona e distruggi una carta sul terreno avversario.</t>
   </si>
   <si>
-    <t>Equipaggia questa carta ad una tua carta edificio. Quando quella carta verrebbe distrutta per effetto di una carta, imposta la sua fede a 10 e scomunica questa carta.</t>
-  </si>
-  <si>
-    <t>Ogni volta che un Token Gub-ner viene evocato sul tuo terreno, distruggilo immediatamente. Per ogni Token Gub-ner distrutto tramite questo effetto, scomunica la prima carta del tuo reliquiario e perdi 3 peccato.</t>
-  </si>
-  <si>
-    <t>Ogni volta che una tua carta viene scomunicata, il tuo avversario riceve 3 peccato.</t>
-  </si>
-  <si>
-    <t>Quando questo santo viene sconfitto o distrutto, scomunicalo. Quando questa carta viene scomunicata puoi prendere fino a 3 carte dalla tua mano e rimetterle nel reliquiario.Poi, pescane altrettante.</t>
-  </si>
-  <si>
-    <t>Dopo il calcolo dei danni, Infliggi gli stessi danni che questa carta riceve al santo avversario attaccante. Se quel santo viene distrutto tramite questo effetto, perdi peccato pari alla fede iniziale di quel santo.</t>
-  </si>
-  <si>
     <t>Cerca nel tuo reliquiario un artefatto. Giocalo sul tuo terreno e scomunica questa carta.</t>
   </si>
   <si>
     <t>Manda una tua carta dalla mano al cimitero. Pesca 3 carte.</t>
   </si>
   <si>
-    <t>Un tuo Santo bersaglio riceve +7 Fede.</t>
-  </si>
-  <si>
-    <t>Due tuoi Santi bersaglio ricevono +6 Fede ciascuno.</t>
-  </si>
-  <si>
     <t>Un tuo Santo bersaglio riceve Fede pari alla sua fede iniziale.</t>
   </si>
   <si>
-    <t>Gioca questa carta solo se il Peccato dell'avversario è pari o inferiore a 50. L'avversario riceve 10 Peccato.</t>
-  </si>
-  <si>
     <t>Assalto</t>
   </si>
   <si>
@@ -1740,9 +1629,6 @@
     <t>Recupero da Cimitero</t>
   </si>
   <si>
-    <t>Scegli fino a 3 carte scomunicate bersaglio, rimettile nel tuo reliquiario e mischialo. Successivamente, se controlli Av'drna o Ph'drna, pesca una carta.</t>
-  </si>
-  <si>
     <t>1/4 (-3)</t>
   </si>
   <si>
@@ -1812,27 +1698,15 @@
     <t>Editto del Faraone</t>
   </si>
   <si>
-    <t>Scegli un artefatto o un edificio avversario. Distruggilo. Poi, ricevi 3 peccato.</t>
-  </si>
-  <si>
     <t>Offerta al Nilo</t>
   </si>
   <si>
-    <t>Manda 1 carta dalla mano al cimitero; pesca 2 carte. Se la carta mandata era un santo, rimuovi 3 peccato.</t>
-  </si>
-  <si>
     <t>Rito di Imbalsamazione Regale</t>
   </si>
   <si>
-    <t>Scegli 1 santo nel tuo cimitero con croci inferiori o uguali a 6; aggiungilo alla mano. Poi, puoi mandare una carta dalla mano al cimitero.</t>
-  </si>
-  <si>
     <t>Guardia del Sarcofago</t>
   </si>
   <si>
-    <t>Una volta per turno, quando subiresti il primo attacco dietto, annullalo. Poi questa carta perte 2 fede. Quando la fede di questa carta diventa pari o inferiore a 0, distrggila.</t>
-  </si>
-  <si>
     <t>Via della Piramide</t>
   </si>
   <si>
@@ -1842,67 +1716,193 @@
     <t>Piaga: Acque di Sangue</t>
   </si>
   <si>
-    <t>Ogni Santo avversario perde 2 Fede. Poi puoi cercare nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario.</t>
-  </si>
-  <si>
     <t>Piaga: Rane Invasive</t>
   </si>
   <si>
-    <t>Infliggi 6 Peccato all'avversario. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
     <t>Piaga delle Locuste</t>
   </si>
   <si>
     <t>Piaga: Tenebre d'Egitto</t>
   </si>
   <si>
-    <t>Durante il prossimo turno dell'avversario, pesca 1 carta in meno (minimo 1). Cerca nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario.</t>
-  </si>
-  <si>
     <t>Piaga: Morte dei Primogeniti</t>
   </si>
   <si>
-    <t>Un Santo avversario perde 6 Fede. Poi infliggi 4 Peccato all'avversario. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
     <t>Piaga: Zanzare del Deserto</t>
   </si>
   <si>
     <t>Piaga: Mosche d'Egitto</t>
   </si>
   <si>
-    <t>Scegli 1 Artefatto o 1 Edificio avversario: distruggilo. Poi puoi cercare nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario.</t>
-  </si>
-  <si>
     <t>Piaga: Ulcere della Carne</t>
   </si>
   <si>
     <t>Piaga: Grandine di Fuoco</t>
   </si>
   <si>
-    <t>Ogni Santo avversario perde 3 Fede. Poi puoi distruggere 1 Artefatto avversario. Poi puoi cercare nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario.</t>
-  </si>
-  <si>
     <t>Piaga: Morte del Bestiame</t>
   </si>
   <si>
-    <t>Scegli un santo sul terreno e distruggilo. Poi infliggi 3 Peccato all'avversario. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
     <t>Una volta per turno, quando questa carta attacca un Santo avversario, puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
   </si>
   <si>
     <t>Portatore delle Piaghe</t>
   </si>
   <si>
-    <t>Ogni Santo avversario perde 3 Fede. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
-    <t>Scegli fino a 2 Santi avversari: ognuno perde 4 Fede. Poi infliggi 2 Peccato all'avversario. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
-  </si>
-  <si>
     <t>Questa carta può essere evocata solo scomunicando 3 carte Piaga dalla tua mano o cimitero, senza pagare costo di Ispirazione. Questa carta non può essere bersagliata dagli effetti di altre carte. Una volta per turno, scegli e attiva un effetto di qualsiasi carta "Piaga" benedizione o maledizione.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un tuo Santo viene distrutto o giochi una carta "Sigillo", aggiungi 1 Segnalino Sigillo su questa carta. Puoi rimuovere un numero di Segnalini Sigillo pari alle Croci di una carta (tua o avversaria) il cui effetto sta per distruggere questa carta: annulla quell'effetto e questa carta non viene distrutta. Quando questa carta lascia il campo, rimuovi tutti i Segnalini Sigillo.</t>
+  </si>
+  <si>
+    <t>All'inizio del tuo turno, ricevi +1 Ispirazione in questo turno.</t>
+  </si>
+  <si>
+    <t>Ogni volta che giochi una Benedizione o una Maledizione, aggiungi 1 Segnalino su questa carta. Puoi rimuovere 3 Segnalini da questa carta: cerca nel tuo reliquiario una Benedizione o Maledizione, rivelala e aggiungila alla tua mano. Poi mischia il reliquiario.</t>
+  </si>
+  <si>
+    <t>Ogni volta che giochi una Benedizione, pesca una carta. Se è un Santo, scomunica quella carta. Se è un Artefatto o Edificio, rimetti quella carta nel tuo reliquiario e mischia. Se è una Benedizione o Maledizione, tienila in mano.</t>
+  </si>
+  <si>
+    <t>Sacrifica un tuo Santo. Quando giochi questa carta, aggiungi la Fede iniziale del Santo sacrificato alla Fede di questa carta. Quando questo Santo viene sconfitto in battaglia o distrutto per effetto di una carta non genera Peccato.</t>
+  </si>
+  <si>
+    <t>Una volta per turno, scegli uno dei seguenti effetti: � Prendi un Santo dal tuo cimitero e aggiungilo alla tua mano, poi distruggi questa carta. � Se non controlli Santi, annulla il primo attacco che ricevi durante il prossimo turno avversario.</t>
+  </si>
+  <si>
+    <t>Ogni volta che peschi una carta, ogni tuo Santo sul campo riceve +2 Fede.</t>
+  </si>
+  <si>
+    <t>Se questo Santo distrugge un Santo con un attacco, torna nella tua mano.</t>
+  </si>
+  <si>
+    <t>Prima della tua fase di pescata, devi distruggere un Santo bersaglio sul campo. Se hai distrutto un tuo Santo, infliggi 2 Peccato all'avversario. Se hai distrutto un Santo avversario, rimuovi 1 Peccato. Se, durante l'attivazione di questo effetto non sono presenti santi sul terreno, distruggi questa carta.</t>
+  </si>
+  <si>
+    <t>Ogni carta "Pietra" distrutta viene messa nel reliquiario del suo proprietario invece che nel cimitero.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un Token Albero viene sconfitto, infliggi 1 Peccato all'avversario.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un Santo avversario attacca, subisce 2 danni. Se un Santo avversario viene distrutto da questo effetto, rimuovi 2 Peccato.</t>
+  </si>
+  <si>
+    <t>Le tue carte Albero non possono essere bersagliate da Maledizioni o Benedizioni avversarie. Se una carta Albero viene scomunicata, viene messa nel reliquiario del suo proprietario invece che nella zona scomunicate.</t>
+  </si>
+  <si>
+    <t>Se questo Santo distrugge un Santo avversario, aumenta la sua Fede di 4.</t>
+  </si>
+  <si>
+    <t>Puoi mandare questa carta dal campo al cimitero: evoca un qualsiasi Santo bersaglio dal tuo cimitero.</t>
+  </si>
+  <si>
+    <t>Puoi giocare questa carta senza pagare il suo costo di Ispirazione. Puoi giocare i Santi dalla tua mano pagando metà del loro costo di Ispirazione (arrotondato per eccesso).</t>
+  </si>
+  <si>
+    <t>Guarda la prima carta del tuo reliquiario. Se è una Benedizione o Maledizione, pescala. Altrimenti, rimischia il reliquiario.</t>
+  </si>
+  <si>
+    <t>Durante la tua fase di pescata, pesca una carta aggiuntiva.</t>
+  </si>
+  <si>
+    <t>Una volta per turno, quando l'avversario pesca una carta, puoi fargli rimischiare quella carta nel reliquiario e pescare di nuovo.</t>
+  </si>
+  <si>
+    <t>Manda un Santo bersaglio dal tuo reliquiario al cimitero. Rimuovi Peccato pari alla Fede e Forza di quel Santo.</t>
+  </si>
+  <si>
+    <t>Scegli 1 Artefatto o 1 Edificio avversario. Distruggilo. Poi ricevi 3 Peccato.</t>
+  </si>
+  <si>
+    <t>Manda 1 carta dalla mano al cimitero; pesca 2 carte. Se la carta mandata era un Santo, rimuovi 3 Peccato.</t>
+  </si>
+  <si>
+    <t>Scegli 1 tuo Santo nel cimitero con Croci pari o inferiori a 6: aggiungilo alla mano. Poi puoi mandare 1 carta dalla tua mano al cimitero.</t>
+  </si>
+  <si>
+    <t>Una volta per turno, quando subiresti il primo attacco diretto, annullalo. Poi questa carta perde 2 Fede. Quando la Fede di questa carta diventa pari o inferiore a 0, distruggila.</t>
+  </si>
+  <si>
+    <t>Ogni volta che l'avversario pesca una carta, questa carta perde 1 Fede e tu rimuovi 2 Peccato. Se la Fede di questa carta diventa 0, distruggi Av'drna.</t>
+  </si>
+  <si>
+    <t>Una volta per turno, puoi attivare l'effetto di questa carta: scomunica la carta in cima al tuo reliquiario.</t>
+  </si>
+  <si>
+    <t>Quando questa carta entra in campo, scegli uno slot Artefatto avversario: quello slot diventa inutilizzabile finche questa carta rimane sul terreno.</t>
+  </si>
+  <si>
+    <t>Scegli fino a 3 carte scomunicate bersaglio, rimettile nel tuo reliquiario e mischialo.Successivamente, se controlli Av'drna o Ph'drna, pesca una carta.</t>
+  </si>
+  <si>
+    <t>Puoi includere questa carta solo in un reliquiario composto interamente da carte con espansione Ph-Dak'Gaph. Ogni volta che peschi una carta, ricevi 1 Peccato. Ogni volta che una carta viene scomunicata, rimuovi 1 Peccato.</t>
+  </si>
+  <si>
+    <t>Equipaggia questa carta a un tuo Edificio. Quando quell'Edificio verrebbe distrutto per effetto di una carta, imposta la sua Fede a 10 e scomunica questa carta.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un Token Gub-ner viene evocato sul tuo terreno, distruggilo immediatamente. Per ogni Token Gub-ner distrutto tramite questo effetto, scomunica la prima carta del tuo reliquiario e rimuovi 3 Peccato.</t>
+  </si>
+  <si>
+    <t>Ogni volta che una tua carta viene scomunicata, il tuo avversario riceve 3 Peccato.</t>
+  </si>
+  <si>
+    <t>Quando questo Santo viene sconfitto o distrutto, scomunicalo. Quando questa carta viene scomunicata, puoi prendere fino a 3 carte dalla tua mano e rimetterle nel reliquiario. Poi, pescane altrettante.</t>
+  </si>
+  <si>
+    <t>Quando questa carta riceve danno da un Santo avversario, quel Santo subisce lo stesso danno. Se quel Santo viene distrutto da questo effetto, rimuovi Peccato pari alla sua Fede iniziale.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un Token o un Santo viene mandato dal campo al cimitero, questo santo riceve +1 Fede e +1 Forza.</t>
+  </si>
+  <si>
+    <t>Una volta per turno, puoi distruggere un tuo Santo bersaglio. Rimuovi Peccato pari alla Fede di quel Santo al momento della distruzione.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un tuo Santo viene mandato al cimitero, evoca un Token Spirito Vacuo sul suo posto.</t>
+  </si>
+  <si>
+    <t>Ogni carta che passa dal tuo campo direttamente al cimitero viene invece aggiunta alla tua mano.</t>
+  </si>
+  <si>
+    <t>Quando questo Santo scende in campo, per ogni 5 carte nel tuo cimitero questa carta riceve +2 Fede e +2 Forza.</t>
+  </si>
+  <si>
+    <t>Un tuo Santo bersaglio riceve +5 Fede.</t>
+  </si>
+  <si>
+    <t>Due tuoi Santi bersaglio ricevono +3 Fede ciascuno.</t>
+  </si>
+  <si>
+    <t>Gioca questa carta solo se il Peccato dell'avversario è pari o inferiore a 50. L'avversario riceve 15 Peccato.</t>
+  </si>
+  <si>
+    <t>Ogni Santo avversario perde 2 Fede. Puoi cercare nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario. Infine infliggi 1 Peccato a te stesso.</t>
+  </si>
+  <si>
+    <t>Infliggi 6 Peccato all'avversario e 1 a te stesso. Puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
+  </si>
+  <si>
+    <t>Durante il prossimo turno dell'avversario, pesca 1 carta in meno (minimo 1). Cerca nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario. Infine infliggi 1 Peccato a te stesso.</t>
+  </si>
+  <si>
+    <t>Un Santo avversario perde 6 Fede. Infliggi 4 Peccato all'avversario e 1 a te stesso. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
+  </si>
+  <si>
+    <t>Ogni Santo avversario perde 3 Fede. Poi puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano. Infine, infliggi 1 Peccato a te stesso.</t>
+  </si>
+  <si>
+    <t>Scegli 1 Artefatto o 1 Edificio avversario: distruggilo. Poi puoi cercare nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario. Infine infliggi 2 Peccato a te stesso.</t>
+  </si>
+  <si>
+    <t>Scegli fino a 2 Santi avversari: ognuno perde 4 Fede. Poi infliggi 3 Peccato all'avversario e 1 a te stesso. Puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
+  </si>
+  <si>
+    <t>Ogni Santo avversario perde 3 Fede. Poi puoi distruggere 1 Artefatto avversario. Puoi cercare nel tuo reliquiario una carta "Piaga", aggiungerla alla tua mano e mischiare il reliquiario. Infine infliggi 2 Peccato a te stesso.</t>
+  </si>
+  <si>
+    <t>Scegli un santo sul terreno e distruggilo. Poi infliggi 3 Peccato all'avversario e 2 a te stesso. Puoi riprendere dal tuo cimitero una carta "Piaga" e aggiungerla alla tua mano.</t>
   </si>
 </sst>
 </file>
@@ -3676,28 +3676,28 @@
         <v>6</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>556</v>
+        <v>519</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>557</v>
+        <v>520</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>558</v>
+        <v>521</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>559</v>
+        <v>522</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>560</v>
+        <v>523</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>561</v>
+        <v>524</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>562</v>
+        <v>525</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>563</v>
+        <v>526</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3705,28 +3705,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>565</v>
+        <v>527</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>567</v>
+        <v>529</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>569</v>
+        <v>531</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>570</v>
+        <v>532</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>571</v>
+        <v>533</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>572</v>
+        <v>534</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3734,28 +3734,28 @@
         <v>103</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>573</v>
+        <v>535</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>567</v>
+        <v>529</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>574</v>
+        <v>536</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>575</v>
+        <v>537</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>571</v>
+        <v>533</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>565</v>
+        <v>527</v>
       </c>
       <c r="I3" s="20" t="s">
-        <v>576</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3763,28 +3763,28 @@
         <v>167</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>578</v>
+        <v>540</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>574</v>
+        <v>536</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>570</v>
+        <v>532</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>576</v>
+        <v>538</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3792,28 +3792,28 @@
         <v>209</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>565</v>
+        <v>527</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>579</v>
+        <v>541</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>580</v>
+        <v>542</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>581</v>
+        <v>543</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>582</v>
+        <v>544</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>583</v>
+        <v>545</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>574</v>
+        <v>536</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3821,28 +3821,28 @@
         <v>246</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>584</v>
+        <v>546</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>580</v>
+        <v>542</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>574</v>
+        <v>536</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>582</v>
+        <v>544</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>568</v>
+        <v>530</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3850,28 +3850,28 @@
         <v>78</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>585</v>
+        <v>547</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>580</v>
+        <v>542</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>586</v>
+        <v>548</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>565</v>
+        <v>527</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>576</v>
+        <v>538</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="14.25" x14ac:dyDescent="0.25">
@@ -3879,28 +3879,28 @@
         <v>271</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>570</v>
+        <v>532</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>566</v>
+        <v>528</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>585</v>
+        <v>547</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>581</v>
+        <v>543</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>574</v>
+        <v>536</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>570</v>
+        <v>532</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>577</v>
+        <v>539</v>
       </c>
       <c r="I8" s="20" t="s">
-        <v>576</v>
+        <v>538</v>
       </c>
     </row>
   </sheetData>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="12" t="s">
-        <v>298</v>
+        <v>568</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>9</v>
@@ -4008,7 +4008,7 @@
         <v>4</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>9</v>
@@ -4027,7 +4027,7 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="12" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>9</v>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="12" t="s">
-        <v>305</v>
+        <v>569</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>9</v>
@@ -4067,7 +4067,7 @@
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="12" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>9</v>
@@ -4088,13 +4088,13 @@
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>314</v>
+        <v>570</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>20</v>
       </c>
@@ -4109,13 +4109,13 @@
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>315</v>
+        <v>571</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>21</v>
       </c>
@@ -4132,7 +4132,7 @@
         <v>3</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>317</v>
+        <v>572</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>9</v>
@@ -4153,13 +4153,13 @@
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="12" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>23</v>
       </c>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>321</v>
+        <v>573</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>9</v>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>325</v>
+        <v>574</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>9</v>
@@ -4214,7 +4214,7 @@
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="12" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>9</v>
@@ -4237,7 +4237,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>338</v>
+        <v>322</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>9</v>
@@ -4260,7 +4260,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>339</v>
+        <v>323</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>9</v>
@@ -4283,7 +4283,7 @@
         <v>10</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>342</v>
+        <v>325</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>9</v>
@@ -4302,7 +4302,7 @@
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>346</v>
+        <v>328</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>9</v>
@@ -4325,7 +4325,7 @@
         <v>3</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>356</v>
+        <v>332</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>9</v>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="E20" s="14"/>
       <c r="F20" s="12" t="s">
-        <v>359</v>
+        <v>335</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>9</v>
@@ -4365,7 +4365,7 @@
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>363</v>
+        <v>339</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>9</v>
@@ -4384,7 +4384,7 @@
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>366</v>
+        <v>341</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>9</v>
@@ -4403,7 +4403,7 @@
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
       <c r="F23" s="12" t="s">
-        <v>367</v>
+        <v>342</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>9</v>
@@ -4422,7 +4422,7 @@
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
       <c r="F24" s="12" t="s">
-        <v>368</v>
+        <v>343</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>9</v>
@@ -4441,7 +4441,7 @@
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
       <c r="F25" s="12" t="s">
-        <v>369</v>
+        <v>344</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>9</v>
@@ -4464,7 +4464,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>370</v>
+        <v>345</v>
       </c>
       <c r="G26" s="7" t="s">
         <v>9</v>
@@ -4487,7 +4487,7 @@
         <v>3</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>371</v>
+        <v>346</v>
       </c>
       <c r="G27" s="7" t="s">
         <v>9</v>
@@ -4506,7 +4506,7 @@
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="12" t="s">
-        <v>372</v>
+        <v>347</v>
       </c>
       <c r="G28" s="7" t="s">
         <v>9</v>
@@ -4525,7 +4525,7 @@
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
       <c r="F29" s="12" t="s">
-        <v>373</v>
+        <v>348</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>9</v>
@@ -4544,7 +4544,7 @@
       <c r="D30" s="14"/>
       <c r="E30" s="14"/>
       <c r="F30" s="12" t="s">
-        <v>374</v>
+        <v>349</v>
       </c>
       <c r="G30" s="7" t="s">
         <v>9</v>
@@ -4567,7 +4567,7 @@
         <v>3</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>377</v>
+        <v>351</v>
       </c>
       <c r="G31" s="7" t="s">
         <v>9</v>
@@ -4590,7 +4590,7 @@
         <v>4</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>381</v>
+        <v>354</v>
       </c>
       <c r="G32" s="7" t="s">
         <v>9</v>
@@ -4613,7 +4613,7 @@
         <v>6</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>400</v>
+        <v>373</v>
       </c>
       <c r="G33" s="7" t="s">
         <v>9</v>
@@ -4632,7 +4632,7 @@
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
       <c r="F34" s="12" t="s">
-        <v>403</v>
+        <v>376</v>
       </c>
       <c r="G34" s="7" t="s">
         <v>9</v>
@@ -4655,7 +4655,7 @@
         <v>0</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>405</v>
+        <v>378</v>
       </c>
       <c r="G35" s="7" t="s">
         <v>9</v>
@@ -4678,7 +4678,7 @@
         <v>2</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>408</v>
+        <v>381</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>9</v>
@@ -4697,7 +4697,7 @@
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
       <c r="F37" s="12" t="s">
-        <v>418</v>
+        <v>391</v>
       </c>
       <c r="G37" s="7" t="s">
         <v>9</v>
@@ -4720,7 +4720,7 @@
         <v>3</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>421</v>
+        <v>394</v>
       </c>
       <c r="G38" s="7" t="s">
         <v>9</v>
@@ -4743,7 +4743,7 @@
         <v>3</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>422</v>
+        <v>395</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>9</v>
@@ -4766,7 +4766,7 @@
         <v>6</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>423</v>
+        <v>396</v>
       </c>
       <c r="G40" s="7" t="s">
         <v>9</v>
@@ -4785,7 +4785,7 @@
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
       <c r="F41" s="12" t="s">
-        <v>426</v>
+        <v>399</v>
       </c>
       <c r="G41" s="7" t="s">
         <v>9</v>
@@ -4804,7 +4804,7 @@
       <c r="D42" s="14"/>
       <c r="E42" s="14"/>
       <c r="F42" s="12" t="s">
-        <v>427</v>
+        <v>400</v>
       </c>
       <c r="G42" s="7" t="s">
         <v>9</v>
@@ -4823,7 +4823,7 @@
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
       <c r="F43" s="12" t="s">
-        <v>444</v>
+        <v>417</v>
       </c>
       <c r="G43" s="7" t="s">
         <v>9</v>
@@ -4846,7 +4846,7 @@
         <v>3</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>446</v>
+        <v>419</v>
       </c>
       <c r="G44" s="7" t="s">
         <v>9</v>
@@ -4865,7 +4865,7 @@
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
       <c r="F45" s="12" t="s">
-        <v>447</v>
+        <v>420</v>
       </c>
       <c r="G45" s="7" t="s">
         <v>9</v>
@@ -4884,7 +4884,7 @@
       <c r="D46" s="14"/>
       <c r="E46" s="14"/>
       <c r="F46" s="12" t="s">
-        <v>448</v>
+        <v>421</v>
       </c>
       <c r="G46" s="7" t="s">
         <v>9</v>
@@ -4907,7 +4907,7 @@
         <v>4</v>
       </c>
       <c r="F47" s="12" t="s">
-        <v>449</v>
+        <v>422</v>
       </c>
       <c r="G47" s="7" t="s">
         <v>9</v>
@@ -4926,7 +4926,7 @@
       <c r="D48" s="14"/>
       <c r="E48" s="14"/>
       <c r="F48" s="12" t="s">
-        <v>450</v>
+        <v>423</v>
       </c>
       <c r="G48" s="7" t="s">
         <v>9</v>
@@ -4945,7 +4945,7 @@
       <c r="D49" s="14"/>
       <c r="E49" s="14"/>
       <c r="F49" s="12" t="s">
-        <v>453</v>
+        <v>426</v>
       </c>
       <c r="G49" s="7" t="s">
         <v>9</v>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="E50" s="14"/>
       <c r="F50" s="12" t="s">
-        <v>459</v>
+        <v>432</v>
       </c>
       <c r="G50" s="7" t="s">
         <v>9</v>
@@ -4985,7 +4985,7 @@
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
       <c r="F51" s="12" t="s">
-        <v>472</v>
+        <v>445</v>
       </c>
       <c r="G51" s="7" t="s">
         <v>9</v>
@@ -5004,7 +5004,7 @@
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
       <c r="F52" s="12" t="s">
-        <v>473</v>
+        <v>446</v>
       </c>
       <c r="G52" s="7" t="s">
         <v>9</v>
@@ -5023,7 +5023,7 @@
       <c r="D53" s="14"/>
       <c r="E53" s="14"/>
       <c r="F53" s="12" t="s">
-        <v>480</v>
+        <v>453</v>
       </c>
       <c r="G53" s="7" t="s">
         <v>9</v>
@@ -5042,7 +5042,7 @@
       <c r="D54" s="14"/>
       <c r="E54" s="14"/>
       <c r="F54" s="12" t="s">
-        <v>486</v>
+        <v>459</v>
       </c>
       <c r="G54" s="7" t="s">
         <v>9</v>
@@ -5061,7 +5061,7 @@
       <c r="D55" s="14"/>
       <c r="E55" s="14"/>
       <c r="F55" s="12" t="s">
-        <v>487</v>
+        <v>460</v>
       </c>
       <c r="G55" s="7" t="s">
         <v>9</v>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="E56" s="14"/>
       <c r="F56" s="12" t="s">
-        <v>503</v>
+        <v>476</v>
       </c>
       <c r="G56" s="7" t="s">
         <v>9</v>
@@ -5101,7 +5101,7 @@
       <c r="D57" s="14"/>
       <c r="E57" s="14"/>
       <c r="F57" s="12" t="s">
-        <v>506</v>
+        <v>479</v>
       </c>
       <c r="G57" s="7" t="s">
         <v>9</v>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="E58" s="14"/>
       <c r="F58" s="12" t="s">
-        <v>512</v>
+        <v>485</v>
       </c>
       <c r="G58" s="7" t="s">
         <v>9</v>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="E59" s="14"/>
       <c r="F59" s="12" t="s">
-        <v>514</v>
+        <v>487</v>
       </c>
       <c r="G59" s="7" t="s">
         <v>9</v>
@@ -5166,7 +5166,7 @@
         <v>3</v>
       </c>
       <c r="F60" s="12" t="s">
-        <v>519</v>
+        <v>492</v>
       </c>
       <c r="G60" s="7" t="s">
         <v>9</v>
@@ -5185,7 +5185,7 @@
       <c r="D61" s="14"/>
       <c r="E61" s="14"/>
       <c r="F61" s="12" t="s">
-        <v>520</v>
+        <v>493</v>
       </c>
       <c r="G61" s="7" t="s">
         <v>9</v>
@@ -5208,7 +5208,7 @@
         <v>5</v>
       </c>
       <c r="F62" s="12" t="s">
-        <v>521</v>
+        <v>494</v>
       </c>
       <c r="G62" s="7" t="s">
         <v>9</v>
@@ -5231,7 +5231,7 @@
         <v>4</v>
       </c>
       <c r="F63" s="12" t="s">
-        <v>522</v>
+        <v>495</v>
       </c>
       <c r="G63" s="7" t="s">
         <v>9</v>
@@ -5250,7 +5250,7 @@
       <c r="D64" s="14"/>
       <c r="E64" s="14"/>
       <c r="F64" s="12" t="s">
-        <v>523</v>
+        <v>496</v>
       </c>
       <c r="G64" s="7" t="s">
         <v>9</v>
@@ -5258,7 +5258,7 @@
     </row>
     <row r="65" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
-        <v>550</v>
+        <v>513</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>18</v>
@@ -5269,13 +5269,13 @@
       <c r="D65" s="14"/>
       <c r="E65" s="14"/>
       <c r="F65" s="12" t="s">
-        <v>551</v>
+        <v>514</v>
       </c>
       <c r="G65" s="7"/>
     </row>
     <row r="66" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A66" s="18" t="s">
-        <v>552</v>
+        <v>515</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>18</v>
@@ -5286,13 +5286,13 @@
       <c r="D66" s="14"/>
       <c r="E66" s="14"/>
       <c r="F66" s="12" t="s">
-        <v>553</v>
+        <v>516</v>
       </c>
       <c r="G66" s="7"/>
     </row>
     <row r="67" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
-        <v>554</v>
+        <v>517</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>18</v>
@@ -5303,7 +5303,7 @@
       <c r="D67" s="14"/>
       <c r="E67" s="14"/>
       <c r="F67" s="12" t="s">
-        <v>555</v>
+        <v>518</v>
       </c>
       <c r="G67" s="7"/>
     </row>
@@ -7372,7 +7372,7 @@
       <c r="D2" s="15"/>
       <c r="E2" s="15"/>
       <c r="F2" s="16" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>78</v>
@@ -7391,7 +7391,7 @@
       <c r="D3" s="15"/>
       <c r="E3" s="15"/>
       <c r="F3" s="16" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>78</v>
@@ -7414,7 +7414,7 @@
         <v>8</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>349</v>
+        <v>329</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>78</v>
@@ -7433,7 +7433,7 @@
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="16" t="s">
-        <v>351</v>
+        <v>330</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>78</v>
@@ -7454,7 +7454,7 @@
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="16" t="s">
-        <v>378</v>
+        <v>352</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>78</v>
@@ -7477,7 +7477,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>379</v>
+        <v>353</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>78</v>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="16" t="s">
-        <v>388</v>
+        <v>361</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>78</v>
@@ -7521,7 +7521,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>389</v>
+        <v>362</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>78</v>
@@ -7544,7 +7544,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>390</v>
+        <v>363</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>78</v>
@@ -7567,7 +7567,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>396</v>
+        <v>369</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>78</v>
@@ -7588,7 +7588,7 @@
       </c>
       <c r="E12" s="15"/>
       <c r="F12" s="16" t="s">
-        <v>402</v>
+        <v>375</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>78</v>
@@ -7609,7 +7609,7 @@
       </c>
       <c r="E13" s="15"/>
       <c r="F13" s="16" t="s">
-        <v>406</v>
+        <v>379</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>78</v>
@@ -7632,7 +7632,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>410</v>
+        <v>383</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>78</v>
@@ -7655,7 +7655,7 @@
         <v>8</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>417</v>
+        <v>390</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>78</v>
@@ -7674,7 +7674,7 @@
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
       <c r="F16" s="16" t="s">
-        <v>456</v>
+        <v>429</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>78</v>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="E17" s="15"/>
       <c r="F17" s="16" t="s">
-        <v>477</v>
+        <v>450</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>78</v>
@@ -7718,7 +7718,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>78</v>
@@ -7741,7 +7741,7 @@
         <v>4</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>490</v>
+        <v>463</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>78</v>
@@ -7764,7 +7764,7 @@
         <v>3</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>499</v>
+        <v>472</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>78</v>
@@ -7787,7 +7787,7 @@
         <v>3</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>499</v>
+        <v>472</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>78</v>
@@ -7806,7 +7806,7 @@
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
       <c r="F22" s="16" t="s">
-        <v>501</v>
+        <v>474</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>78</v>
@@ -7829,7 +7829,7 @@
         <v>8</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>507</v>
+        <v>480</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>78</v>
@@ -7850,7 +7850,7 @@
       </c>
       <c r="E24" s="15"/>
       <c r="F24" s="16" t="s">
-        <v>517</v>
+        <v>490</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>78</v>
@@ -7871,7 +7871,7 @@
       </c>
       <c r="E25" s="15"/>
       <c r="F25" s="12" t="s">
-        <v>531</v>
+        <v>503</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>78</v>
@@ -8982,7 +8982,7 @@
         <v>3</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>103</v>
@@ -9005,7 +9005,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>103</v>
@@ -9028,7 +9028,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>103</v>
@@ -9051,7 +9051,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>103</v>
@@ -9074,7 +9074,7 @@
         <v>3</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>103</v>
@@ -9097,7 +9097,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>103</v>
@@ -9120,7 +9120,7 @@
         <v>8</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>302</v>
+        <v>575</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>103</v>
@@ -9141,7 +9141,7 @@
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>322</v>
+        <v>576</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>103</v>
@@ -9162,7 +9162,7 @@
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="12" t="s">
-        <v>323</v>
+        <v>577</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>103</v>
@@ -9179,7 +9179,7 @@
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
       <c r="F11" s="12" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>103</v>
@@ -9198,7 +9198,7 @@
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>103</v>
@@ -9219,7 +9219,7 @@
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>103</v>
@@ -9242,7 +9242,7 @@
         <v>4</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>103</v>
@@ -9263,7 +9263,7 @@
       </c>
       <c r="E15" s="14"/>
       <c r="F15" s="12" t="s">
-        <v>336</v>
+        <v>578</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>103</v>
@@ -9282,7 +9282,7 @@
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="12" t="s">
-        <v>341</v>
+        <v>324</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>103</v>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="E17" s="14"/>
       <c r="F17" s="12" t="s">
-        <v>350</v>
+        <v>579</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>103</v>
@@ -9322,13 +9322,13 @@
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>352</v>
+        <v>331</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>121</v>
       </c>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="E19" s="14"/>
       <c r="F19" s="12" t="s">
-        <v>354</v>
+        <v>580</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>103</v>
@@ -9366,7 +9366,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>375</v>
+        <v>581</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>103</v>
@@ -9387,7 +9387,7 @@
       </c>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>382</v>
+        <v>355</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>103</v>
@@ -9410,7 +9410,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>383</v>
+        <v>356</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>103</v>
@@ -9433,7 +9433,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>384</v>
+        <v>357</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>103</v>
@@ -9452,7 +9452,7 @@
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
       <c r="F24" s="12" t="s">
-        <v>385</v>
+        <v>358</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>103</v>
@@ -9475,7 +9475,7 @@
         <v>1</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>392</v>
+        <v>365</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>103</v>
@@ -9494,7 +9494,7 @@
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
       <c r="F26" s="12" t="s">
-        <v>393</v>
+        <v>366</v>
       </c>
       <c r="G26" s="7" t="s">
         <v>103</v>
@@ -9513,7 +9513,7 @@
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
       <c r="F27" s="12" t="s">
-        <v>404</v>
+        <v>377</v>
       </c>
       <c r="G27" s="7" t="s">
         <v>103</v>
@@ -9532,7 +9532,7 @@
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="12" t="s">
-        <v>407</v>
+        <v>380</v>
       </c>
       <c r="G28" s="7" t="s">
         <v>103</v>
@@ -9555,7 +9555,7 @@
         <v>2</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>412</v>
+        <v>385</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>103</v>
@@ -9578,7 +9578,7 @@
         <v>2</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>416</v>
+        <v>389</v>
       </c>
       <c r="G30" s="7" t="s">
         <v>103</v>
@@ -9601,7 +9601,7 @@
         <v>3</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>431</v>
+        <v>404</v>
       </c>
       <c r="G31" s="7" t="s">
         <v>103</v>
@@ -9620,7 +9620,7 @@
       <c r="D32" s="14"/>
       <c r="E32" s="14"/>
       <c r="F32" s="12" t="s">
-        <v>432</v>
+        <v>405</v>
       </c>
       <c r="G32" s="7" t="s">
         <v>103</v>
@@ -9643,7 +9643,7 @@
         <v>4</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>433</v>
+        <v>406</v>
       </c>
       <c r="G33" s="7" t="s">
         <v>103</v>
@@ -9666,7 +9666,7 @@
         <v>6</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>434</v>
+        <v>407</v>
       </c>
       <c r="G34" s="7" t="s">
         <v>103</v>
@@ -9685,7 +9685,7 @@
       <c r="D35" s="14"/>
       <c r="E35" s="14"/>
       <c r="F35" s="12" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="G35" s="7" t="s">
         <v>103</v>
@@ -9706,7 +9706,7 @@
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="12" t="s">
-        <v>436</v>
+        <v>409</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>103</v>
@@ -9725,7 +9725,7 @@
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
       <c r="F37" s="12" t="s">
-        <v>437</v>
+        <v>410</v>
       </c>
       <c r="G37" s="7" t="s">
         <v>103</v>
@@ -9744,7 +9744,7 @@
       <c r="D38" s="14"/>
       <c r="E38" s="14"/>
       <c r="F38" s="12" t="s">
-        <v>438</v>
+        <v>411</v>
       </c>
       <c r="G38" s="7" t="s">
         <v>103</v>
@@ -9763,7 +9763,7 @@
       <c r="D39" s="14"/>
       <c r="E39" s="14"/>
       <c r="F39" s="12" t="s">
-        <v>439</v>
+        <v>412</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>103</v>
@@ -9782,7 +9782,7 @@
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
       <c r="F40" s="12" t="s">
-        <v>445</v>
+        <v>418</v>
       </c>
       <c r="G40" s="7" t="s">
         <v>103</v>
@@ -9801,7 +9801,7 @@
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
       <c r="F41" s="12" t="s">
-        <v>450</v>
+        <v>423</v>
       </c>
       <c r="G41" s="7" t="s">
         <v>103</v>
@@ -9822,7 +9822,7 @@
       </c>
       <c r="E42" s="14"/>
       <c r="F42" s="12" t="s">
-        <v>455</v>
+        <v>428</v>
       </c>
       <c r="G42" s="7" t="s">
         <v>103</v>
@@ -9843,7 +9843,7 @@
       </c>
       <c r="E43" s="14"/>
       <c r="F43" s="12" t="s">
-        <v>467</v>
+        <v>440</v>
       </c>
       <c r="G43" s="7" t="s">
         <v>103</v>
@@ -9864,7 +9864,7 @@
       </c>
       <c r="E44" s="14"/>
       <c r="F44" s="12" t="s">
-        <v>468</v>
+        <v>441</v>
       </c>
       <c r="G44" s="7" t="s">
         <v>103</v>
@@ -9883,7 +9883,7 @@
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
       <c r="F45" s="12" t="s">
-        <v>476</v>
+        <v>449</v>
       </c>
       <c r="G45" s="7" t="s">
         <v>103</v>
@@ -9904,7 +9904,7 @@
       </c>
       <c r="E46" s="14"/>
       <c r="F46" s="12" t="s">
-        <v>481</v>
+        <v>454</v>
       </c>
       <c r="G46" s="7" t="s">
         <v>103</v>
@@ -9927,7 +9927,7 @@
         <v>4</v>
       </c>
       <c r="F47" s="12" t="s">
-        <v>483</v>
+        <v>456</v>
       </c>
       <c r="G47" s="7" t="s">
         <v>103</v>
@@ -9946,7 +9946,7 @@
       <c r="D48" s="14"/>
       <c r="E48" s="14"/>
       <c r="F48" s="12" t="s">
-        <v>495</v>
+        <v>468</v>
       </c>
       <c r="G48" s="7" t="s">
         <v>103</v>
@@ -9969,7 +9969,7 @@
         <v>2</v>
       </c>
       <c r="F49" s="12" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="G49" s="7" t="s">
         <v>103</v>
@@ -9992,7 +9992,7 @@
         <v>4</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>497</v>
+        <v>470</v>
       </c>
       <c r="G50" s="7" t="s">
         <v>103</v>
@@ -10011,7 +10011,7 @@
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
       <c r="F51" s="12" t="s">
-        <v>500</v>
+        <v>473</v>
       </c>
       <c r="G51" s="7" t="s">
         <v>103</v>
@@ -10030,7 +10030,7 @@
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
       <c r="F52" s="12" t="s">
-        <v>504</v>
+        <v>477</v>
       </c>
       <c r="G52" s="7" t="s">
         <v>103</v>
@@ -10049,7 +10049,7 @@
       <c r="D53" s="14"/>
       <c r="E53" s="14"/>
       <c r="F53" s="12" t="s">
-        <v>505</v>
+        <v>478</v>
       </c>
       <c r="G53" s="7" t="s">
         <v>103</v>
@@ -10068,7 +10068,7 @@
       <c r="D54" s="14"/>
       <c r="E54" s="14"/>
       <c r="F54" s="12" t="s">
-        <v>508</v>
+        <v>481</v>
       </c>
       <c r="G54" s="7" t="s">
         <v>103</v>
@@ -10089,7 +10089,7 @@
         <v>8</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>494</v>
+        <v>467</v>
       </c>
       <c r="G55" s="7" t="s">
         <v>103</v>
@@ -10110,7 +10110,7 @@
         <v>0</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>494</v>
+        <v>467</v>
       </c>
       <c r="G56" s="7" t="s">
         <v>103</v>
@@ -10129,7 +10129,7 @@
       <c r="D57" s="14"/>
       <c r="E57" s="14"/>
       <c r="F57" s="12" t="s">
-        <v>510</v>
+        <v>483</v>
       </c>
       <c r="G57" s="7" t="s">
         <v>103</v>
@@ -10152,7 +10152,7 @@
         <v>0</v>
       </c>
       <c r="F58" s="12" t="s">
-        <v>511</v>
+        <v>484</v>
       </c>
       <c r="G58" s="7" t="s">
         <v>103</v>
@@ -10171,7 +10171,7 @@
       <c r="D59" s="14"/>
       <c r="E59" s="14"/>
       <c r="F59" s="12" t="s">
-        <v>516</v>
+        <v>489</v>
       </c>
       <c r="G59" s="7" t="s">
         <v>103</v>
@@ -10190,7 +10190,7 @@
       <c r="D60" s="14"/>
       <c r="E60" s="14"/>
       <c r="F60" s="12" t="s">
-        <v>526</v>
+        <v>498</v>
       </c>
       <c r="G60" s="7" t="s">
         <v>103</v>
@@ -10213,7 +10213,7 @@
         <v>15</v>
       </c>
       <c r="F61" s="12" t="s">
-        <v>528</v>
+        <v>500</v>
       </c>
       <c r="G61" s="7" t="s">
         <v>103</v>
@@ -11225,13 +11225,13 @@
         <v>1</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>301</v>
+        <v>582</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>168</v>
       </c>
@@ -11248,7 +11248,7 @@
         <v>15</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>308</v>
+        <v>583</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>167</v>
@@ -11267,7 +11267,7 @@
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
       <c r="F4" s="12" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>167</v>
@@ -11290,7 +11290,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>167</v>
@@ -11313,7 +11313,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>340</v>
+        <v>584</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>167</v>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="12" t="s">
-        <v>347</v>
+        <v>585</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>167</v>
@@ -11355,7 +11355,7 @@
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>348</v>
+        <v>586</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>167</v>
@@ -11378,7 +11378,7 @@
         <v>4</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>362</v>
+        <v>338</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>167</v>
@@ -11399,7 +11399,7 @@
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="12" t="s">
-        <v>364</v>
+        <v>340</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>167</v>
@@ -11422,7 +11422,7 @@
         <v>5</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>386</v>
+        <v>359</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>167</v>
@@ -11441,7 +11441,7 @@
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>401</v>
+        <v>374</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>167</v>
@@ -11460,7 +11460,7 @@
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>409</v>
+        <v>382</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>167</v>
@@ -11483,7 +11483,7 @@
         <v>3</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>413</v>
+        <v>386</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>167</v>
@@ -11506,7 +11506,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>414</v>
+        <v>387</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>167</v>
@@ -11527,7 +11527,7 @@
       </c>
       <c r="E16" s="14"/>
       <c r="F16" s="12" t="s">
-        <v>415</v>
+        <v>388</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>167</v>
@@ -11546,7 +11546,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="16" t="s">
-        <v>419</v>
+        <v>392</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>167</v>
@@ -11569,7 +11569,7 @@
         <v>10</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>420</v>
+        <v>393</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>167</v>
@@ -11588,7 +11588,7 @@
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="12" t="s">
-        <v>425</v>
+        <v>398</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>167</v>
@@ -11607,7 +11607,7 @@
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
       <c r="F20" s="12" t="s">
-        <v>430</v>
+        <v>403</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>167</v>
@@ -11628,7 +11628,7 @@
       </c>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>440</v>
+        <v>413</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>167</v>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>440</v>
+        <v>413</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>167</v>
@@ -11670,7 +11670,7 @@
       </c>
       <c r="E23" s="14"/>
       <c r="F23" s="12" t="s">
-        <v>440</v>
+        <v>413</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>167</v>
@@ -11689,7 +11689,7 @@
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
       <c r="F24" s="12" t="s">
-        <v>450</v>
+        <v>423</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>167</v>
@@ -11712,7 +11712,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>452</v>
+        <v>425</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>167</v>
@@ -11735,7 +11735,7 @@
         <v>20</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>454</v>
+        <v>427</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>167</v>
@@ -11754,7 +11754,7 @@
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
       <c r="F27" s="12" t="s">
-        <v>462</v>
+        <v>435</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>167</v>
@@ -11777,7 +11777,7 @@
         <v>1</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>470</v>
+        <v>443</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>167</v>
@@ -11800,7 +11800,7 @@
         <v>2</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>471</v>
+        <v>444</v>
       </c>
       <c r="G29" s="8" t="s">
         <v>167</v>
@@ -11823,7 +11823,7 @@
         <v>2</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>478</v>
+        <v>451</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>167</v>
@@ -11846,7 +11846,7 @@
         <v>2</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>479</v>
+        <v>452</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>167</v>
@@ -11869,7 +11869,7 @@
         <v>2</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>484</v>
+        <v>457</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>167</v>
@@ -11892,7 +11892,7 @@
         <v>6</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>485</v>
+        <v>458</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>167</v>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="E34" s="14"/>
       <c r="F34" s="12" t="s">
-        <v>488</v>
+        <v>461</v>
       </c>
       <c r="G34" s="8" t="s">
         <v>167</v>
@@ -11932,7 +11932,7 @@
       <c r="D35" s="14"/>
       <c r="E35" s="14"/>
       <c r="F35" s="12" t="s">
-        <v>502</v>
+        <v>475</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>167</v>
@@ -11953,7 +11953,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>494</v>
+        <v>467</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>167</v>
@@ -11972,7 +11972,7 @@
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
       <c r="F37" s="12" t="s">
-        <v>513</v>
+        <v>486</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>167</v>
@@ -11995,7 +11995,7 @@
         <v>2</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>515</v>
+        <v>488</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>167</v>
@@ -12016,7 +12016,7 @@
       </c>
       <c r="E39" s="14"/>
       <c r="F39" s="12" t="s">
-        <v>518</v>
+        <v>491</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>167</v>
@@ -12035,7 +12035,7 @@
       <c r="D40" s="8"/>
       <c r="E40" s="8"/>
       <c r="F40" s="12" t="s">
-        <v>533</v>
+        <v>587</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>167</v>
@@ -12054,7 +12054,7 @@
       <c r="D41" s="8"/>
       <c r="E41" s="8"/>
       <c r="F41" s="12" t="s">
-        <v>534</v>
+        <v>505</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>167</v>
@@ -12073,7 +12073,7 @@
       <c r="D42" s="8"/>
       <c r="E42" s="8"/>
       <c r="F42" s="12" t="s">
-        <v>535</v>
+        <v>506</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>167</v>
@@ -12081,7 +12081,7 @@
     </row>
     <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>587</v>
+        <v>549</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>15</v>
@@ -12100,7 +12100,7 @@
     </row>
     <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>589</v>
+        <v>550</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>18</v>
@@ -12111,7 +12111,7 @@
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
       <c r="F44" s="12" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>167</v>
@@ -12119,7 +12119,7 @@
     </row>
     <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>591</v>
+        <v>551</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>18</v>
@@ -12130,7 +12130,7 @@
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
       <c r="F45" s="12" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>167</v>
@@ -12138,7 +12138,7 @@
     </row>
     <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>593</v>
+        <v>552</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>8</v>
@@ -12151,7 +12151,7 @@
       </c>
       <c r="E46" s="8"/>
       <c r="F46" s="12" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="G46" s="8" t="s">
         <v>167</v>
@@ -12159,7 +12159,7 @@
     </row>
     <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>595</v>
+        <v>553</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>18</v>
@@ -12170,7 +12170,7 @@
       <c r="D47" s="8"/>
       <c r="E47" s="8"/>
       <c r="F47" s="12" t="s">
-        <v>596</v>
+        <v>554</v>
       </c>
       <c r="G47" s="8" t="s">
         <v>167</v>
@@ -12178,18 +12178,18 @@
     </row>
     <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>597</v>
+        <v>555</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C48" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8"/>
       <c r="F48" s="12" t="s">
-        <v>598</v>
+        <v>610</v>
       </c>
       <c r="G48" s="8" t="s">
         <v>167</v>
@@ -12197,18 +12197,18 @@
     </row>
     <row r="49" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>599</v>
+        <v>556</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C49" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8"/>
       <c r="F49" s="12" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>167</v>
@@ -12216,7 +12216,7 @@
     </row>
     <row r="50" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>601</v>
+        <v>557</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>13</v>
@@ -12231,7 +12231,7 @@
         <v>6</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>614</v>
+        <v>565</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>167</v>
@@ -12239,18 +12239,18 @@
     </row>
     <row r="51" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>602</v>
+        <v>558</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C51" s="8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8"/>
       <c r="F51" s="12" t="s">
-        <v>603</v>
+        <v>612</v>
       </c>
       <c r="G51" s="8" t="s">
         <v>167</v>
@@ -12258,18 +12258,18 @@
     </row>
     <row r="52" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>604</v>
+        <v>559</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C52" s="8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8"/>
       <c r="F52" s="12" t="s">
-        <v>605</v>
+        <v>613</v>
       </c>
       <c r="G52" s="8" t="s">
         <v>167</v>
@@ -12277,18 +12277,18 @@
     </row>
     <row r="53" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>606</v>
+        <v>560</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C53" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8"/>
       <c r="F53" s="12" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>167</v>
@@ -12296,18 +12296,18 @@
     </row>
     <row r="54" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>607</v>
+        <v>561</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C54" s="8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
       <c r="F54" s="12" t="s">
-        <v>608</v>
+        <v>615</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>167</v>
@@ -12315,18 +12315,18 @@
     </row>
     <row r="55" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>609</v>
+        <v>562</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C55" s="8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
       <c r="F55" s="12" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G55" s="8" t="s">
         <v>167</v>
@@ -12334,18 +12334,18 @@
     </row>
     <row r="56" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
-        <v>610</v>
+        <v>563</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C56" s="8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
       <c r="F56" s="12" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>167</v>
@@ -12353,18 +12353,18 @@
     </row>
     <row r="57" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
-        <v>612</v>
+        <v>564</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C57" s="8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D57" s="8"/>
       <c r="E57" s="8"/>
       <c r="F57" s="12" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>167</v>
@@ -12372,7 +12372,7 @@
     </row>
     <row r="58" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
-        <v>615</v>
+        <v>566</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>13</v>
@@ -12387,7 +12387,7 @@
         <v>10</v>
       </c>
       <c r="F58" s="12" t="s">
-        <v>618</v>
+        <v>567</v>
       </c>
       <c r="G58" s="8" t="s">
         <v>167</v>
@@ -12458,7 +12458,7 @@
       </c>
       <c r="E2" s="14"/>
       <c r="F2" s="12" t="s">
-        <v>309</v>
+        <v>592</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>209</v>
@@ -12494,7 +12494,7 @@
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
       <c r="F3" s="12" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>209</v>
@@ -12530,7 +12530,7 @@
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
       <c r="F4" s="12" t="s">
-        <v>343</v>
+        <v>326</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>209</v>
@@ -12566,7 +12566,7 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="12" t="s">
-        <v>344</v>
+        <v>327</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>209</v>
@@ -12604,7 +12604,7 @@
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="12" t="s">
-        <v>355</v>
+        <v>593</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>209</v>
@@ -12644,7 +12644,7 @@
         <v>5</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>357</v>
+        <v>333</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>209</v>
@@ -12680,7 +12680,7 @@
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>358</v>
+        <v>334</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>209</v>
@@ -12716,7 +12716,7 @@
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>361</v>
+        <v>337</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>209</v>
@@ -12754,7 +12754,7 @@
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="12" t="s">
-        <v>365</v>
+        <v>594</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>209</v>
@@ -12794,7 +12794,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>376</v>
+        <v>350</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>209</v>
@@ -12834,7 +12834,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>391</v>
+        <v>364</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>209</v>
@@ -12872,7 +12872,7 @@
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>394</v>
+        <v>367</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>209</v>
@@ -12912,7 +12912,7 @@
         <v>7</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>395</v>
+        <v>368</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>209</v>
@@ -12948,7 +12948,7 @@
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="12" t="s">
-        <v>398</v>
+        <v>371</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>209</v>
@@ -12988,7 +12988,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>399</v>
+        <v>372</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>209</v>
@@ -13024,7 +13024,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="12" t="s">
-        <v>424</v>
+        <v>397</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>209</v>
@@ -13062,7 +13062,7 @@
       </c>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>428</v>
+        <v>401</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>209</v>
@@ -13098,7 +13098,7 @@
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="12" t="s">
-        <v>429</v>
+        <v>402</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>209</v>
@@ -13138,7 +13138,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>441</v>
+        <v>414</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>209</v>
@@ -13174,7 +13174,7 @@
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>442</v>
+        <v>415</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>209</v>
@@ -13210,7 +13210,7 @@
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>450</v>
+        <v>423</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>209</v>
@@ -13246,7 +13246,7 @@
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
       <c r="F23" s="12" t="s">
-        <v>461</v>
+        <v>434</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>209</v>
@@ -13282,7 +13282,7 @@
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
       <c r="F24" s="12" t="s">
-        <v>564</v>
+        <v>595</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>209</v>
@@ -13322,7 +13322,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>469</v>
+        <v>442</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>209</v>
@@ -13358,7 +13358,7 @@
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
       <c r="F26" s="12" t="s">
-        <v>491</v>
+        <v>464</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>209</v>
@@ -13396,7 +13396,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>494</v>
+        <v>467</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>209</v>
@@ -13430,7 +13430,7 @@
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="12" t="s">
-        <v>525</v>
+        <v>596</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>209</v>
@@ -13470,7 +13470,7 @@
         <v>4</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>530</v>
+        <v>502</v>
       </c>
       <c r="G29" s="8" t="s">
         <v>209</v>
@@ -13510,7 +13510,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>532</v>
+        <v>504</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>209</v>
@@ -13548,7 +13548,7 @@
       </c>
       <c r="E31" s="8"/>
       <c r="F31" s="13" t="s">
-        <v>536</v>
+        <v>507</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>209</v>
@@ -13584,7 +13584,7 @@
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
       <c r="F32" s="13" t="s">
-        <v>537</v>
+        <v>597</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>209</v>
@@ -13622,7 +13622,7 @@
       </c>
       <c r="E33" s="8"/>
       <c r="F33" s="13" t="s">
-        <v>538</v>
+        <v>598</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>209</v>
@@ -13660,7 +13660,7 @@
       </c>
       <c r="E34" s="8"/>
       <c r="F34" s="13" t="s">
-        <v>539</v>
+        <v>599</v>
       </c>
       <c r="G34" s="8" t="s">
         <v>209</v>
@@ -13700,7 +13700,7 @@
         <v>6</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>540</v>
+        <v>600</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>209</v>
@@ -13740,7 +13740,7 @@
         <v>3</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>541</v>
+        <v>601</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>209</v>
@@ -13776,7 +13776,7 @@
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
       <c r="F37" s="13" t="s">
-        <v>542</v>
+        <v>508</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>209</v>
@@ -19403,7 +19403,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>292</v>
+        <v>602</v>
       </c>
       <c r="G2" s="11" t="s">
         <v>246</v>
@@ -19426,7 +19426,7 @@
         <v>3</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>246</v>
@@ -19447,7 +19447,7 @@
       </c>
       <c r="E4" s="14"/>
       <c r="F4" s="12" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>246</v>
@@ -19470,7 +19470,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>246</v>
@@ -19491,7 +19491,7 @@
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="12" t="s">
-        <v>324</v>
+        <v>603</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>246</v>
@@ -19512,7 +19512,7 @@
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="12" t="s">
-        <v>345</v>
+        <v>604</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>246</v>
@@ -19533,7 +19533,7 @@
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>353</v>
+        <v>605</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>246</v>
@@ -19552,7 +19552,7 @@
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>360</v>
+        <v>336</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>246</v>
@@ -19575,7 +19575,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>380</v>
+        <v>606</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>246</v>
@@ -19598,7 +19598,7 @@
         <v>4</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>387</v>
+        <v>360</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>246</v>
@@ -19617,7 +19617,7 @@
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>397</v>
+        <v>370</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>246</v>
@@ -19634,7 +19634,7 @@
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>451</v>
+        <v>424</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>246</v>
@@ -19653,7 +19653,7 @@
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="12" t="s">
-        <v>457</v>
+        <v>430</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>246</v>
@@ -19672,7 +19672,7 @@
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="12" t="s">
-        <v>465</v>
+        <v>438</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>246</v>
@@ -19691,7 +19691,7 @@
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="12" t="s">
-        <v>466</v>
+        <v>439</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>246</v>
@@ -19710,7 +19710,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="12" t="s">
-        <v>474</v>
+        <v>447</v>
       </c>
       <c r="G17" s="11" t="s">
         <v>246</v>
@@ -19729,7 +19729,7 @@
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="G18" s="11" t="s">
         <v>246</v>
@@ -19752,7 +19752,7 @@
         <v>6</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>492</v>
+        <v>465</v>
       </c>
       <c r="G19" s="11" t="s">
         <v>246</v>
@@ -19773,7 +19773,7 @@
       </c>
       <c r="E20" s="14"/>
       <c r="F20" s="12" t="s">
-        <v>493</v>
+        <v>466</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>246</v>
@@ -19794,7 +19794,7 @@
       </c>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>494</v>
+        <v>467</v>
       </c>
       <c r="G21" s="11" t="s">
         <v>246</v>
@@ -19813,7 +19813,7 @@
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>498</v>
+        <v>471</v>
       </c>
       <c r="G22" s="11" t="s">
         <v>246</v>
@@ -19834,7 +19834,7 @@
       </c>
       <c r="E23" s="14"/>
       <c r="F23" s="12" t="s">
-        <v>509</v>
+        <v>482</v>
       </c>
       <c r="G23" s="11" t="s">
         <v>246</v>
@@ -19857,7 +19857,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>527</v>
+        <v>499</v>
       </c>
       <c r="G24" s="11" t="s">
         <v>246</v>
@@ -19878,7 +19878,7 @@
       </c>
       <c r="E25" s="14"/>
       <c r="F25" s="12" t="s">
-        <v>529</v>
+        <v>501</v>
       </c>
       <c r="G25" s="11" t="s">
         <v>246</v>
@@ -22475,7 +22475,7 @@
       <c r="D2" s="14"/>
       <c r="E2" s="14"/>
       <c r="F2" s="12" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>271</v>
@@ -22494,7 +22494,7 @@
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
       <c r="F3" s="12" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>271</v>
@@ -22513,7 +22513,7 @@
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
       <c r="F4" s="12" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>271</v>
@@ -22532,7 +22532,7 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="12" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>271</v>
@@ -22551,7 +22551,7 @@
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="12" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>271</v>
@@ -22570,7 +22570,7 @@
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="12" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>271</v>
@@ -22589,7 +22589,7 @@
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>544</v>
+        <v>607</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>271</v>
@@ -22608,7 +22608,7 @@
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>545</v>
+        <v>608</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>271</v>
@@ -22627,7 +22627,7 @@
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
       <c r="F10" s="12" t="s">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>271</v>
@@ -22646,7 +22646,7 @@
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
       <c r="F11" s="12" t="s">
-        <v>543</v>
+        <v>509</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>271</v>
@@ -22665,7 +22665,7 @@
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>411</v>
+        <v>384</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>271</v>
@@ -22684,7 +22684,7 @@
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>546</v>
+        <v>510</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>271</v>
@@ -22703,7 +22703,7 @@
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="12" t="s">
-        <v>443</v>
+        <v>416</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>271</v>
@@ -22722,7 +22722,7 @@
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="12" t="s">
-        <v>458</v>
+        <v>431</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>271</v>
@@ -22741,7 +22741,7 @@
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="12" t="s">
-        <v>460</v>
+        <v>433</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>271</v>
@@ -22760,7 +22760,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="12" t="s">
-        <v>463</v>
+        <v>436</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>271</v>
@@ -22779,7 +22779,7 @@
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>464</v>
+        <v>437</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>271</v>
@@ -22802,7 +22802,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>482</v>
+        <v>455</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>271</v>
@@ -22821,7 +22821,7 @@
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
       <c r="F20" s="12" t="s">
-        <v>547</v>
+        <v>609</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>271</v>
@@ -22840,7 +22840,7 @@
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>524</v>
+        <v>497</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>271</v>
@@ -22848,7 +22848,7 @@
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>548</v>
+        <v>511</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>15</v>
@@ -22859,7 +22859,7 @@
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>549</v>
+        <v>512</v>
       </c>
       <c r="G22" s="8"/>
     </row>

</xml_diff>

<commit_message>
fix summon condition di Dio
</commit_message>
<xml_diff>
--- a/Holy War.xlsx
+++ b/Holy War.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\Holy-War-Python-Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A5464C-CE41-4223-B4F5-E83F3AAD71ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA50BF36-E102-4B2C-8FD3-AA144E0147A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="8" r:id="rId1"/>
@@ -4280,7 +4280,7 @@
         <v>25</v>
       </c>
       <c r="E17" s="14">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>325</v>

</xml_diff>